<commit_message>
Initial commit: anemia pen cloud app
</commit_message>
<xml_diff>
--- a/labels.xlsx
+++ b/labels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alna7\Downloads\anemiaapp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3BE5B30-805E-4A90-BF4C-F1D0F70654D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D1886D-6FC7-47A0-81C0-D5E4C025CEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>GENDER</t>
   </si>
   <si>
-    <t>image_path</t>
-  </si>
-  <si>
     <t>hb</t>
   </si>
   <si>
@@ -501,6 +498,9 @@
   </si>
   <si>
     <t>Age</t>
+  </si>
+  <si>
+    <t>filename</t>
   </si>
 </sst>
 </file>
@@ -1377,16 +1377,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
@@ -1394,7 +1394,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2">
         <v>9.3000000000000007</v>
@@ -1403,12 +1403,12 @@
         <v>82</v>
       </c>
       <c r="E2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>10.199999999999999</v>
@@ -1417,12 +1417,12 @@
         <v>77</v>
       </c>
       <c r="E3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>10.7</v>
@@ -1431,12 +1431,12 @@
         <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>11.7</v>
@@ -1445,12 +1445,12 @@
         <v>73</v>
       </c>
       <c r="E5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>11.6</v>
@@ -1459,12 +1459,12 @@
         <v>74</v>
       </c>
       <c r="E6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>15</v>
@@ -1473,12 +1473,12 @@
         <v>77</v>
       </c>
       <c r="E7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>12</v>
@@ -1487,12 +1487,12 @@
         <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9">
         <v>14.3</v>
@@ -1501,12 +1501,12 @@
         <v>84</v>
       </c>
       <c r="E9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10">
         <v>9.8000000000000007</v>
@@ -1515,12 +1515,12 @@
         <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>12.2</v>
@@ -1529,12 +1529,12 @@
         <v>70</v>
       </c>
       <c r="E11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12">
         <v>12</v>
@@ -1543,12 +1543,12 @@
         <v>81</v>
       </c>
       <c r="E12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -1557,12 +1557,12 @@
         <v>88</v>
       </c>
       <c r="E13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>10.5</v>
@@ -1571,12 +1571,12 @@
         <v>82</v>
       </c>
       <c r="E14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15">
         <v>11.4</v>
@@ -1585,12 +1585,12 @@
         <v>65</v>
       </c>
       <c r="E15" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16">
         <v>13.3</v>
@@ -1599,12 +1599,12 @@
         <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17">
         <v>13.5</v>
@@ -1613,12 +1613,12 @@
         <v>55</v>
       </c>
       <c r="E17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18">
         <v>11</v>
@@ -1627,12 +1627,12 @@
         <v>78</v>
       </c>
       <c r="E18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <v>11.8</v>
@@ -1641,12 +1641,12 @@
         <v>77</v>
       </c>
       <c r="E19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>11</v>
@@ -1655,12 +1655,12 @@
         <v>65</v>
       </c>
       <c r="E20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21">
         <v>13.6</v>
@@ -1669,12 +1669,12 @@
         <v>30</v>
       </c>
       <c r="E21" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22">
         <v>9.8000000000000007</v>
@@ -1683,12 +1683,12 @@
         <v>46</v>
       </c>
       <c r="E22" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23">
         <v>12.6</v>
@@ -1697,12 +1697,12 @@
         <v>65</v>
       </c>
       <c r="E23" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24">
         <v>9.6</v>
@@ -1711,12 +1711,12 @@
         <v>57</v>
       </c>
       <c r="E24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25">
         <v>9.1999999999999993</v>
@@ -1725,12 +1725,12 @@
         <v>56</v>
       </c>
       <c r="E25" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26">
         <v>8.6999999999999993</v>
@@ -1739,12 +1739,12 @@
         <v>53</v>
       </c>
       <c r="E26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27">
         <v>8.6</v>
@@ -1753,12 +1753,12 @@
         <v>60</v>
       </c>
       <c r="E27" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28">
         <v>9.4</v>
@@ -1767,12 +1767,12 @@
         <v>59</v>
       </c>
       <c r="E28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29">
         <v>15.5</v>
@@ -1781,12 +1781,12 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30">
         <v>10.9</v>
@@ -1795,12 +1795,12 @@
         <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31">
         <v>12.7</v>
@@ -1809,12 +1809,12 @@
         <v>70</v>
       </c>
       <c r="E31" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32">
         <v>14.8</v>
@@ -1823,12 +1823,12 @@
         <v>54</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B33">
         <v>14.1</v>
@@ -1837,12 +1837,12 @@
         <v>40</v>
       </c>
       <c r="E33" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34">
         <v>13.9</v>
@@ -1851,12 +1851,12 @@
         <v>34</v>
       </c>
       <c r="E34" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35">
         <v>14.1</v>
@@ -1865,12 +1865,12 @@
         <v>53</v>
       </c>
       <c r="E35" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36">
         <v>15.7</v>
@@ -1879,12 +1879,12 @@
         <v>36</v>
       </c>
       <c r="E36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37">
         <v>13.9</v>
@@ -1893,12 +1893,12 @@
         <v>51</v>
       </c>
       <c r="E37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38">
         <v>13.6</v>
@@ -1907,12 +1907,12 @@
         <v>51</v>
       </c>
       <c r="E38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39">
         <v>15.4</v>
@@ -1921,12 +1921,12 @@
         <v>56</v>
       </c>
       <c r="E39" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B40">
         <v>13.7</v>
@@ -1935,12 +1935,12 @@
         <v>47</v>
       </c>
       <c r="E40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B41">
         <v>13.3</v>
@@ -1949,12 +1949,12 @@
         <v>46</v>
       </c>
       <c r="E41" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42">
         <v>13.9</v>
@@ -1963,12 +1963,12 @@
         <v>36</v>
       </c>
       <c r="E42" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B43">
         <v>15</v>
@@ -1977,12 +1977,12 @@
         <v>49</v>
       </c>
       <c r="E43" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44">
         <v>14.7</v>
@@ -1991,12 +1991,12 @@
         <v>59</v>
       </c>
       <c r="E44" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B45">
         <v>15.4</v>
@@ -2005,12 +2005,12 @@
         <v>26</v>
       </c>
       <c r="E45" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46">
         <v>14.9</v>
@@ -2019,12 +2019,12 @@
         <v>50</v>
       </c>
       <c r="E46" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B47">
         <v>14.1</v>
@@ -2033,12 +2033,12 @@
         <v>58</v>
       </c>
       <c r="E47" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48">
         <v>14.1</v>
@@ -2047,12 +2047,12 @@
         <v>20</v>
       </c>
       <c r="E48" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B49">
         <v>16.100000000000001</v>
@@ -2061,12 +2061,12 @@
         <v>29</v>
       </c>
       <c r="E49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B50">
         <v>15.1</v>
@@ -2075,12 +2075,12 @@
         <v>33</v>
       </c>
       <c r="E50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B51">
         <v>15.3</v>
@@ -2089,12 +2089,12 @@
         <v>40</v>
       </c>
       <c r="E51" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B52">
         <v>13.9</v>
@@ -2103,12 +2103,12 @@
         <v>54</v>
       </c>
       <c r="E52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B53">
         <v>14.4</v>
@@ -2117,12 +2117,12 @@
         <v>24</v>
       </c>
       <c r="E53" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B54">
         <v>15.1</v>
@@ -2131,12 +2131,12 @@
         <v>43</v>
       </c>
       <c r="E54" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B55">
         <v>15.3</v>
@@ -2145,12 +2145,12 @@
         <v>42</v>
       </c>
       <c r="E55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B56">
         <v>16.899999999999999</v>
@@ -2159,12 +2159,12 @@
         <v>34</v>
       </c>
       <c r="E56" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B57">
         <v>13.2</v>
@@ -2173,12 +2173,12 @@
         <v>24</v>
       </c>
       <c r="E57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B58">
         <v>13.5</v>
@@ -2187,12 +2187,12 @@
         <v>51</v>
       </c>
       <c r="E58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B59">
         <v>15</v>
@@ -2201,12 +2201,12 @@
         <v>56</v>
       </c>
       <c r="E59" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B60">
         <v>15.5</v>
@@ -2215,12 +2215,12 @@
         <v>62</v>
       </c>
       <c r="E60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B61">
         <v>15.6</v>
@@ -2229,12 +2229,12 @@
         <v>41</v>
       </c>
       <c r="E61" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B62">
         <v>15</v>
@@ -2243,12 +2243,12 @@
         <v>50</v>
       </c>
       <c r="E62" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B63">
         <v>13</v>
@@ -2257,12 +2257,12 @@
         <v>40</v>
       </c>
       <c r="E63" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B64">
         <v>14.9</v>
@@ -2271,12 +2271,12 @@
         <v>54</v>
       </c>
       <c r="E64" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B65">
         <v>17.399999999999999</v>
@@ -2285,12 +2285,12 @@
         <v>52</v>
       </c>
       <c r="E65" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B66">
         <v>13.8</v>
@@ -2299,12 +2299,12 @@
         <v>63</v>
       </c>
       <c r="E66" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B67">
         <v>15.9</v>
@@ -2313,12 +2313,12 @@
         <v>55</v>
       </c>
       <c r="E67" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B68">
         <v>16.2</v>
@@ -2327,12 +2327,12 @@
         <v>48</v>
       </c>
       <c r="E68" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B69">
         <v>15.5</v>
@@ -2341,12 +2341,12 @@
         <v>55</v>
       </c>
       <c r="E69" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B70">
         <v>14.1</v>
@@ -2355,12 +2355,12 @@
         <v>51</v>
       </c>
       <c r="E70" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B71">
         <v>15.3</v>
@@ -2369,12 +2369,12 @@
         <v>37</v>
       </c>
       <c r="E71" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B72">
         <v>13.7</v>
@@ -2383,12 +2383,12 @@
         <v>20</v>
       </c>
       <c r="E72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B73">
         <v>13.4</v>
@@ -2397,12 +2397,12 @@
         <v>48</v>
       </c>
       <c r="E73" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B74">
         <v>12.3</v>
@@ -2411,12 +2411,12 @@
         <v>56</v>
       </c>
       <c r="E74" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B75">
         <v>12.9</v>
@@ -2425,12 +2425,12 @@
         <v>48</v>
       </c>
       <c r="E75" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B76">
         <v>13.5</v>
@@ -2439,12 +2439,12 @@
         <v>48</v>
       </c>
       <c r="E76" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B77">
         <v>13.7</v>
@@ -2453,12 +2453,12 @@
         <v>48</v>
       </c>
       <c r="E77" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B78">
         <v>16.8</v>
@@ -2467,12 +2467,12 @@
         <v>60</v>
       </c>
       <c r="E78" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B79">
         <v>15.4</v>
@@ -2481,12 +2481,12 @@
         <v>25</v>
       </c>
       <c r="E79" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B80">
         <v>14.7</v>
@@ -2495,12 +2495,12 @@
         <v>31</v>
       </c>
       <c r="E80" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B81">
         <v>13.5</v>
@@ -2509,12 +2509,12 @@
         <v>40</v>
       </c>
       <c r="E81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B82">
         <v>15.6</v>
@@ -2523,12 +2523,12 @@
         <v>64</v>
       </c>
       <c r="E82" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B83">
         <v>14.8</v>
@@ -2537,12 +2537,12 @@
         <v>24</v>
       </c>
       <c r="E83" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B84">
         <v>14.8</v>
@@ -2551,12 +2551,12 @@
         <v>25</v>
       </c>
       <c r="E84" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B85">
         <v>14.9</v>
@@ -2565,12 +2565,12 @@
         <v>46</v>
       </c>
       <c r="E85" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B86">
         <v>12.4</v>
@@ -2579,12 +2579,12 @@
         <v>42</v>
       </c>
       <c r="E86" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B87">
         <v>16.899999999999999</v>
@@ -2593,12 +2593,12 @@
         <v>48</v>
       </c>
       <c r="E87" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B88">
         <v>15.6</v>
@@ -2607,12 +2607,12 @@
         <v>51</v>
       </c>
       <c r="E88" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B89">
         <v>13.7</v>
@@ -2621,12 +2621,12 @@
         <v>38</v>
       </c>
       <c r="E89" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B90">
         <v>15.4</v>
@@ -2635,12 +2635,12 @@
         <v>44</v>
       </c>
       <c r="E90" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B91">
         <v>13</v>
@@ -2649,12 +2649,12 @@
         <v>21</v>
       </c>
       <c r="E91" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B92">
         <v>15.4</v>
@@ -2663,12 +2663,12 @@
         <v>41</v>
       </c>
       <c r="E92" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B93">
         <v>12.3</v>
@@ -2677,12 +2677,12 @@
         <v>52</v>
       </c>
       <c r="E93" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B94">
         <v>15.2</v>
@@ -2691,12 +2691,12 @@
         <v>34</v>
       </c>
       <c r="E94" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B95">
         <v>13.8</v>
@@ -2705,12 +2705,12 @@
         <v>31</v>
       </c>
       <c r="E95" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B96">
         <v>14.7</v>
@@ -2719,12 +2719,12 @@
         <v>45</v>
       </c>
       <c r="E96" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B97">
         <v>15.1</v>
@@ -2733,12 +2733,12 @@
         <v>49</v>
       </c>
       <c r="E97" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B98">
         <v>15.2</v>
@@ -2747,12 +2747,12 @@
         <v>54</v>
       </c>
       <c r="E98" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B99">
         <v>15.5</v>
@@ -2761,12 +2761,12 @@
         <v>44</v>
       </c>
       <c r="E99" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B100">
         <v>14.5</v>
@@ -2775,12 +2775,12 @@
         <v>63</v>
       </c>
       <c r="E100" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B101">
         <v>14</v>
@@ -2789,12 +2789,12 @@
         <v>28</v>
       </c>
       <c r="E101" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B102">
         <v>15.8</v>
@@ -2803,12 +2803,12 @@
         <v>40</v>
       </c>
       <c r="E102" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B103">
         <v>14.1</v>
@@ -2817,12 +2817,12 @@
         <v>59</v>
       </c>
       <c r="E103" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B104">
         <v>16.5</v>
@@ -2831,12 +2831,12 @@
         <v>45</v>
       </c>
       <c r="E104" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B105">
         <v>7</v>
@@ -2845,12 +2845,12 @@
         <v>26</v>
       </c>
       <c r="E105" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B106">
         <v>15.5</v>
@@ -2859,12 +2859,12 @@
         <v>68</v>
       </c>
       <c r="E106" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B107">
         <v>13</v>
@@ -2873,12 +2873,12 @@
         <v>40</v>
       </c>
       <c r="E107" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B108">
         <v>13.5</v>
@@ -2887,12 +2887,12 @@
         <v>21</v>
       </c>
       <c r="E108" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B109">
         <v>15.7</v>
@@ -2901,12 +2901,12 @@
         <v>59</v>
       </c>
       <c r="E109" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B110">
         <v>15.8</v>
@@ -2915,12 +2915,12 @@
         <v>45</v>
       </c>
       <c r="E110" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B111">
         <v>13.1</v>
@@ -2929,12 +2929,12 @@
         <v>37</v>
       </c>
       <c r="E111" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B112">
         <v>15.4</v>
@@ -2943,12 +2943,12 @@
         <v>57</v>
       </c>
       <c r="E112" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B113">
         <v>14</v>
@@ -2957,12 +2957,12 @@
         <v>58</v>
       </c>
       <c r="E113" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B114">
         <v>15.1</v>
@@ -2971,12 +2971,12 @@
         <v>39</v>
       </c>
       <c r="E114" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B115">
         <v>15.4</v>
@@ -2985,12 +2985,12 @@
         <v>43</v>
       </c>
       <c r="E115" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B116">
         <v>13.7</v>
@@ -2999,12 +2999,12 @@
         <v>28</v>
       </c>
       <c r="E116" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B117">
         <v>15.1</v>
@@ -3013,12 +3013,12 @@
         <v>47</v>
       </c>
       <c r="E117" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B118">
         <v>15.2</v>
@@ -3027,12 +3027,12 @@
         <v>48</v>
       </c>
       <c r="E118" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B119">
         <v>16.7</v>
@@ -3041,12 +3041,12 @@
         <v>41</v>
       </c>
       <c r="E119" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B120">
         <v>15.4</v>
@@ -3055,12 +3055,12 @@
         <v>22</v>
       </c>
       <c r="E120" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B121">
         <v>12.8</v>
@@ -3069,12 +3069,12 @@
         <v>40</v>
       </c>
       <c r="E121" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B122">
         <v>15.7</v>
@@ -3083,12 +3083,12 @@
         <v>33</v>
       </c>
       <c r="E122" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B123">
         <v>15.6</v>
@@ -3097,12 +3097,12 @@
         <v>48</v>
       </c>
       <c r="E123" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B124">
         <v>12.2</v>
@@ -3111,12 +3111,12 @@
         <v>29</v>
       </c>
       <c r="E124" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B125">
         <v>8</v>
@@ -3125,12 +3125,12 @@
         <v>36</v>
       </c>
       <c r="E125" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B126">
         <v>10.7</v>
@@ -3139,12 +3139,12 @@
         <v>30</v>
       </c>
       <c r="E126" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B127">
         <v>8.3000000000000007</v>
@@ -3153,12 +3153,12 @@
         <v>39</v>
       </c>
       <c r="E127" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B128">
         <v>7.8</v>
@@ -3167,12 +3167,12 @@
         <v>29</v>
       </c>
       <c r="E128" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B129">
         <v>11.8</v>
@@ -3181,12 +3181,12 @@
         <v>55</v>
       </c>
       <c r="E129" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B130">
         <v>9.1999999999999993</v>
@@ -3195,12 +3195,12 @@
         <v>27</v>
       </c>
       <c r="E130" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B131">
         <v>13</v>
@@ -3209,12 +3209,12 @@
         <v>32</v>
       </c>
       <c r="E131" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B132">
         <v>11.5</v>
@@ -3223,12 +3223,12 @@
         <v>32</v>
       </c>
       <c r="E132" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B133">
         <v>11.3</v>
@@ -3237,12 +3237,12 @@
         <v>35</v>
       </c>
       <c r="E133" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B134">
         <v>13.2</v>
@@ -3251,12 +3251,12 @@
         <v>38</v>
       </c>
       <c r="E134" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B135">
         <v>10.6</v>
@@ -3265,12 +3265,12 @@
         <v>75</v>
       </c>
       <c r="E135" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B136">
         <v>10.6</v>
@@ -3279,12 +3279,12 @@
         <v>71</v>
       </c>
       <c r="E136" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B137">
         <v>9.1</v>
@@ -3293,12 +3293,12 @@
         <v>29</v>
       </c>
       <c r="E137" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B138">
         <v>10.9</v>
@@ -3307,12 +3307,12 @@
         <v>30</v>
       </c>
       <c r="E138" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B139">
         <v>8.9</v>
@@ -3321,12 +3321,12 @@
         <v>37</v>
       </c>
       <c r="E139" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B140">
         <v>11.5</v>
@@ -3335,12 +3335,12 @@
         <v>57</v>
       </c>
       <c r="E140" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B141">
         <v>10.1</v>
@@ -3349,12 +3349,12 @@
         <v>32</v>
       </c>
       <c r="E141" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B142">
         <v>12.6</v>
@@ -3363,12 +3363,12 @@
         <v>21</v>
       </c>
       <c r="E142" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B143">
         <v>11.9</v>
@@ -3377,12 +3377,12 @@
         <v>21</v>
       </c>
       <c r="E143" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B144">
         <v>14.8</v>
@@ -3391,12 +3391,12 @@
         <v>21</v>
       </c>
       <c r="E144" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B145">
         <v>10.7</v>
@@ -3405,12 +3405,12 @@
         <v>21</v>
       </c>
       <c r="E145" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B146">
         <v>9.8000000000000007</v>
@@ -3419,12 +3419,12 @@
         <v>21</v>
       </c>
       <c r="E146" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B147">
         <v>13.4</v>
@@ -3433,12 +3433,12 @@
         <v>23</v>
       </c>
       <c r="E147" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B148">
         <v>9.1999999999999993</v>
@@ -3447,12 +3447,12 @@
         <v>30</v>
       </c>
       <c r="E148" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B149">
         <v>7.6</v>
@@ -3461,12 +3461,12 @@
         <v>39</v>
       </c>
       <c r="E149" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B150">
         <v>12.2</v>
@@ -3475,7 +3475,7 @@
         <v>48</v>
       </c>
       <c r="E150" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>